<commit_message>
test(register): add register e2e ui tests
Refs: #2
</commit_message>
<xml_diff>
--- a/docs/tests-inventories/0001_auth-inventory.xlsx
+++ b/docs/tests-inventories/0001_auth-inventory.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="01-login-inventory" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="66">
   <si>
     <t xml:space="preserve">Spec ID</t>
   </si>
@@ -68,139 +68,157 @@
     <t xml:space="preserve">DONE</t>
   </si>
   <si>
+    <t xml:space="preserve">AUTH-L-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User session persists after page refresh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authenticated user cannot access login page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login fails with an error message when password is incorrect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login fails with an error message when email does not exist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login fails with an error message when both email &amp; password are incorrect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged out when authentication token is expired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App crash when token is expired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple rapid login attempts do not trigger multiple authentication requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login successfully with special chars password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login successfully with spaces in password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
     <t xml:space="preserve">AUTH-02</t>
   </si>
   <si>
-    <t xml:space="preserve">AUTH-L-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User session persists after page refresh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regression</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authenticated user cannot access login page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login fails with an error message when password is incorrect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Negative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login fails with an error message when email does not exist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login fails with an error message when both email &amp; password are incorrect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User is logged out when authentication token is expired</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extended</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App crash when token is expired</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multiple rapid login attempts do not trigger multiple authentication requests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login successfully with special chars password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login successfully with spaces in password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criticity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-R-01</t>
+    <t xml:space="preserve">AUTH-R-0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with valid credentials login user</t>
   </si>
   <si>
     <t xml:space="preserve">register.spec.ts</t>
   </si>
   <si>
-    <t xml:space="preserve">🔴 High</t>
-  </si>
-  <si>
     <t xml:space="preserve">E2E</t>
   </si>
   <si>
-    <t xml:space="preserve">❌</t>
+    <t xml:space="preserve">Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register fails with existing username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register fails with existing email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register fails with existing username &amp; email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to register without username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to register without email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to register without password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authenticated user cannot access register page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with leading space in the username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-2001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with leading space in the email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with leading space in the password</t>
   </si>
 </sst>
 </file>
@@ -328,7 +346,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="26.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.42"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1018" min="8" style="1" width="11.52"/>
@@ -389,19 +407,19 @@
     </row>
     <row r="3" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>13</v>
@@ -412,19 +430,19 @@
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>13</v>
@@ -435,19 +453,19 @@
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>13</v>
@@ -458,19 +476,19 @@
     </row>
     <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>13</v>
@@ -481,19 +499,19 @@
     </row>
     <row r="7" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>13</v>
@@ -504,45 +522,45 @@
     </row>
     <row r="8" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>13</v>
@@ -553,19 +571,19 @@
     </row>
     <row r="10" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
@@ -576,19 +594,19 @@
     </row>
     <row r="11" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>13</v>
@@ -613,83 +631,351 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P1048576"/>
+  <dimension ref="A1:Q1048576"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="26.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="21.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.67"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="11" style="1" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="112.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="21.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="16.67"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="12" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
[#2] Add register E2E UI tests (#5)
* test(register): add register e2e ui tests

Refs: #2

* test(auth): changes after review

Refs: #2

---------

Co-authored-by: idembele70 <idembele70@gmail>
</commit_message>
<xml_diff>
--- a/docs/tests-inventories/0001_auth-inventory.xlsx
+++ b/docs/tests-inventories/0001_auth-inventory.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="01-login-inventory" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="66">
   <si>
     <t xml:space="preserve">Spec ID</t>
   </si>
@@ -68,139 +68,157 @@
     <t xml:space="preserve">DONE</t>
   </si>
   <si>
+    <t xml:space="preserve">AUTH-L-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User session persists after page refresh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authenticated user cannot access login page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login fails with an error message when password is incorrect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login fails with an error message when email does not exist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login fails with an error message when both email &amp; password are incorrect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged out when authentication token is expired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App crash when token is expired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple rapid login attempts do not trigger multiple authentication requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login successfully with special chars password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-L-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login successfully with spaces in password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
     <t xml:space="preserve">AUTH-02</t>
   </si>
   <si>
-    <t xml:space="preserve">AUTH-L-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User session persists after page refresh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regression</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authenticated user cannot access login page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login fails with an error message when password is incorrect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Negative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login fails with an error message when email does not exist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login fails with an error message when both email &amp; password are incorrect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User is logged out when authentication token is expired</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extended</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App crash when token is expired</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multiple rapid login attempts do not trigger multiple authentication requests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login successfully with special chars password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-L-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login successfully with spaces in password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criticity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTH-R-01</t>
+    <t xml:space="preserve">AUTH-R-0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with valid credentials login user</t>
   </si>
   <si>
     <t xml:space="preserve">register.spec.ts</t>
   </si>
   <si>
-    <t xml:space="preserve">🔴 High</t>
-  </si>
-  <si>
     <t xml:space="preserve">E2E</t>
   </si>
   <si>
-    <t xml:space="preserve">❌</t>
+    <t xml:space="preserve">Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register fails with existing username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register fails with existing email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register fails with existing username &amp; email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to register without username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to register without email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to register without password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authenticated user cannot access register page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with leading space in the username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-2001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with leading space in the email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-R-2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register with leading space in the password</t>
   </si>
 </sst>
 </file>
@@ -328,7 +346,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="26.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.42"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1018" min="8" style="1" width="11.52"/>
@@ -389,19 +407,19 @@
     </row>
     <row r="3" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>13</v>
@@ -412,19 +430,19 @@
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>13</v>
@@ -435,19 +453,19 @@
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>13</v>
@@ -458,19 +476,19 @@
     </row>
     <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>13</v>
@@ -481,19 +499,19 @@
     </row>
     <row r="7" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>13</v>
@@ -504,45 +522,45 @@
     </row>
     <row r="8" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>13</v>
@@ -553,19 +571,19 @@
     </row>
     <row r="10" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
@@ -576,19 +594,19 @@
     </row>
     <row r="11" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>13</v>
@@ -613,83 +631,351 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P1048576"/>
+  <dimension ref="A1:Q1048576"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="26.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="21.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.67"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="11" style="1" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="112.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="21.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="16.67"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="12" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>